<commit_message>
Keep numeric amount and price-unit fields distinct from SAP identifiers
</commit_message>
<xml_diff>
--- a/public/sap-reporting/expansion-150-downloads/EXT-CO17-01.xlsx
+++ b/public/sap-reporting/expansion-150-downloads/EXT-CO17-01.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Layout" sheetId="1" r:id="Ra45ab57daf2549dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flat input" sheetId="2" r:id="Rc7c0ee9e494e499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R5295d3fc0fa54f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Layout" sheetId="1" r:id="Re8461385829b48d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flat input" sheetId="2" r:id="R7762055a6f0a4f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" r:id="R4d0257111d5644f1"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>